<commit_message>
Fase 3B, item 7 (revisão): segundo tenant com roadmap, arquivo e assistente em dois quick wins
Construtora de demonstração: patrocinador do tenant seleciona e decide;
uma oportunidade vai ao roadmap e outra é arquivada, com motivo; um quick
win volta ao roadmap na implantação e é substituído; o assistente do
Jurídico fica em dois quick wins ativos e cada execução conta em um só;
janelas com aviso de duração e volume diferentes. Relatórios regenerados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015mqTFtP1jGUbbpXgao4Nue
</commit_message>
<xml_diff>
--- a/docs/fase-3b/relatorios-construtora/portfolio-oportunidades.xlsx
+++ b/docs/fase-3b/relatorios-construtora/portfolio-oportunidades.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="92">
   <si>
     <t>Área</t>
   </si>
@@ -56,6 +56,9 @@
     <t>Situação</t>
   </si>
   <si>
+    <t>Motivo</t>
+  </si>
+  <si>
     <t>Quick win</t>
   </si>
   <si>
@@ -101,10 +104,13 @@
     <t>selecionada</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>em implantação</t>
   </si>
   <si>
-    <t>Só precisa da base de conhecimento; nenhum assistente.</t>
+    <t>Selecionada de novo, com o procedimento revisado.</t>
   </si>
   <si>
     <t>Obras</t>
@@ -212,6 +218,12 @@
     <t>8 editais por mês</t>
   </si>
   <si>
+    <t>arquivada</t>
+  </si>
+  <si>
+    <t>As licitações passam a ser feitas por uma assessoria externa.</t>
+  </si>
+  <si>
     <t>Engenharia</t>
   </si>
   <si>
@@ -230,10 +242,13 @@
     <t>40 boletins por mês</t>
   </si>
   <si>
-    <t>identificada</t>
-  </si>
-  <si>
-    <t>Devolvida ao portfólio: Depende do novo padrão de medição, que sai em dezembro. (nota anterior 33,3)</t>
+    <t>33,3</t>
+  </si>
+  <si>
+    <t>enviada ao roadmap</t>
+  </si>
+  <si>
+    <t>Depende do novo padrão de medição e de integração com o sistema dos empreiteiros: projeto, não quick win.</t>
   </si>
   <si>
     <t>Portfólio de oportunidades: Construtora Horizonte (demonstração)</t>
@@ -653,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -665,11 +680,11 @@
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="17" customWidth="1"/>
+    <col min="13" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -718,305 +733,326 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" t="s">
+        <v>30</v>
+      </c>
+      <c r="P2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" t="s">
         <v>23</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H3" t="s">
         <v>24</v>
       </c>
-      <c r="J2" t="s">
+      <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
         <v>25</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s">
+        <v>40</v>
+      </c>
+      <c r="N3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P3" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" t="s">
+        <v>49</v>
+      </c>
+      <c r="N4" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" t="s">
         <v>24</v>
       </c>
-      <c r="L2" t="s">
+      <c r="I5" t="s">
         <v>26</v>
       </c>
-      <c r="M2" t="s">
+      <c r="J5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>25</v>
+      </c>
+      <c r="M5" t="s">
+        <v>58</v>
+      </c>
+      <c r="N5" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P5" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" t="s">
         <v>27</v>
       </c>
-      <c r="N2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O2" t="s">
-        <v>29</v>
-      </c>
-      <c r="P2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="I6" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L6" t="s">
         <v>25</v>
       </c>
-      <c r="J3" t="s">
+      <c r="M6" t="s">
+        <v>58</v>
+      </c>
+      <c r="N6" t="s">
+        <v>68</v>
+      </c>
+      <c r="O6" t="s">
+        <v>69</v>
+      </c>
+      <c r="P6" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
         <v>24</v>
       </c>
-      <c r="K3" t="s">
+      <c r="J7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" t="s">
         <v>24</v>
       </c>
-      <c r="L3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M3" t="s">
-        <v>38</v>
-      </c>
-      <c r="N3" t="s">
-        <v>28</v>
-      </c>
-      <c r="O3" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="L7" t="s">
         <v>25</v>
       </c>
-      <c r="J4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L4" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" t="s">
-        <v>47</v>
-      </c>
-      <c r="N4" t="s">
-        <v>28</v>
-      </c>
-      <c r="O4" t="s">
-        <v>39</v>
-      </c>
-      <c r="P4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G5" t="s">
-        <v>55</v>
-      </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J5" t="s">
-        <v>37</v>
-      </c>
-      <c r="K5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" t="s">
-        <v>24</v>
-      </c>
-      <c r="M5" t="s">
-        <v>56</v>
-      </c>
-      <c r="N5" t="s">
-        <v>57</v>
-      </c>
-      <c r="O5" t="s">
-        <v>58</v>
-      </c>
-      <c r="P5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="M7" t="s">
+        <v>76</v>
+      </c>
+      <c r="N7" t="s">
+        <v>77</v>
+      </c>
+      <c r="O7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P7" t="s">
         <v>60</v>
       </c>
-      <c r="B6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L6" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" t="s">
-        <v>56</v>
-      </c>
-      <c r="N6" t="s">
-        <v>57</v>
-      </c>
-      <c r="O6" t="s">
-        <v>58</v>
-      </c>
-      <c r="P6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" t="s">
-        <v>55</v>
-      </c>
-      <c r="H7" t="s">
-        <v>58</v>
-      </c>
-      <c r="I7" t="s">
-        <v>58</v>
-      </c>
-      <c r="J7" t="s">
-        <v>58</v>
-      </c>
-      <c r="K7" t="s">
-        <v>58</v>
-      </c>
-      <c r="L7" t="s">
-        <v>58</v>
-      </c>
-      <c r="M7" t="s">
-        <v>58</v>
-      </c>
-      <c r="N7" t="s">
-        <v>72</v>
-      </c>
-      <c r="O7" t="s">
-        <v>58</v>
-      </c>
-      <c r="P7" t="s">
-        <v>73</v>
+      <c r="Q7" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1036,26 +1072,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1066,10 +1102,10 @@
         <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1080,10 +1116,10 @@
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D6" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1094,10 +1130,10 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1108,10 +1144,10 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1122,10 +1158,10 @@
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>